<commit_message>
Add filtered quotes Excel export feature
</commit_message>
<xml_diff>
--- a/Quote.xlsx
+++ b/Quote.xlsx
@@ -441,77 +441,77 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alexandre Dumas fils</t>
+          <t>J.K. Rowling</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alfred Tennyson</t>
+          <t>Marilyn Monroe</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Allen Saunders</t>
+          <t>Mark Twain</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>André Gide</t>
+          <t>Dr. Seuss</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ayn Rand</t>
+          <t>C.S. Lewis</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bob Marley</t>
+          <t>Jane Austen</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C.S. Lewis</t>
+          <t>Bob Marley</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Charles Bukowski</t>
+          <t>Eleanor Roosevelt</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -521,47 +521,47 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Charles M. Schulz</t>
+          <t>Charles Bukowski</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Douglas Adams</t>
+          <t>Suzanne Collins</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dr. Seuss</t>
+          <t>George R.R. Martin</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>E.E. Cummings</t>
+          <t>Mother Teresa</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Eleanor Roosevelt</t>
+          <t>Ralph Waldo Emerson</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -571,27 +571,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Elie Wiesel</t>
+          <t>Ernest Hemingway</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ernest Hemingway</t>
+          <t>Alexandre Dumas fils</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Friedrich Nietzsche</t>
+          <t>Ayn Rand</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -601,7 +601,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Garrison Keillor</t>
+          <t>Alfred Tennyson</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -611,7 +611,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>George Bernard Shaw</t>
+          <t>Garrison Keillor</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -621,7 +621,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>George Carlin</t>
+          <t>Friedrich Nietzsche</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -631,7 +631,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>George Eliot</t>
+          <t>Elie Wiesel</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -641,17 +641,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>George R.R. Martin</t>
+          <t>E.E. Cummings</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Harper Lee</t>
+          <t>Douglas Adams</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -661,7 +661,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Haruki Murakami</t>
+          <t>André Gide</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -671,7 +671,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Helen Keller</t>
+          <t>Allen Saunders</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -681,7 +681,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>J.D. Salinger</t>
+          <t>Charles M. Schulz</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -691,17 +691,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>J.K. Rowling</t>
+          <t>J.D. Salinger</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>J.M. Barrie</t>
+          <t>Helen Keller</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -721,7 +721,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>James Baldwin</t>
+          <t>George Bernard Shaw</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -731,17 +731,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Jane Austen</t>
+          <t>Harper Lee</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jim Henson</t>
+          <t>Haruki Murakami</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -751,7 +751,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jimi Hendrix</t>
+          <t>George Carlin</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -761,7 +761,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>John Lennon</t>
+          <t>George Eliot</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -771,7 +771,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jorge Luis Borges</t>
+          <t>John Lennon</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -781,7 +781,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Khaled Hosseini</t>
+          <t>Jimi Hendrix</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -791,7 +791,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Madeleine L'Engle</t>
+          <t>Jim Henson</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -801,27 +801,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Marilyn Monroe</t>
+          <t>James Baldwin</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mark Twain</t>
+          <t>J.M. Barrie</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Martin Luther King Jr.</t>
+          <t>Khaled Hosseini</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -831,17 +831,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mother Teresa</t>
+          <t>Madeleine L'Engle</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Pablo Neruda</t>
+          <t>Jorge Luis Borges</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -851,17 +851,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ralph Waldo Emerson</t>
+          <t>Pablo Neruda</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Stephenie Meyer</t>
+          <t>Martin Luther King Jr.</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -871,7 +871,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Steve Martin</t>
+          <t>Stephenie Meyer</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -881,11 +881,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Suzanne Collins</t>
+          <t>Steve Martin</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">

</xml_diff>